<commit_message>
new env and new parsing
</commit_message>
<xml_diff>
--- a/data/input/ЭКСПЕРТ.xlsx
+++ b/data/input/ЭКСПЕРТ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AI Projects\RelayProtection\rza_calculator\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9C67361-F865-4761-8DE8-F7CDFE1EF3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFFD6252-BB5E-4E5E-BE88-752BEE1F4473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="4680" windowWidth="38400" windowHeight="15345" tabRatio="781" activeTab="3" xr2:uid="{F50B1136-9C70-43B5-86FC-BA6162992F35}"/>
+    <workbookView xWindow="0" yWindow="3510" windowWidth="38400" windowHeight="15345" tabRatio="781" xr2:uid="{00F6B97D-33F9-4CAC-A846-B7596DE47128}"/>
   </bookViews>
   <sheets>
     <sheet name="Провода" sheetId="11" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <author>Shkliar</author>
   </authors>
   <commentList>
-    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{7F951C2F-1EA0-4313-8315-1013BAF48BBD}">
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{62D88977-2D99-45CE-9420-333065370904}">
       <text>
         <r>
           <rPr>
@@ -3070,6 +3070,19 @@
       <charset val="204"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Cyr"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Cyr"/>
+      <charset val="204"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
       <color theme="9" tint="-0.249977111117893"/>
@@ -3080,19 +3093,6 @@
       <b/>
       <sz val="10"/>
       <color rgb="FF7030A0"/>
-      <name val="Arial Cyr"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Cyr"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial Cyr"/>
       <charset val="204"/>
     </font>
@@ -3375,6 +3375,69 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -3395,6 +3458,50 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -3437,113 +3544,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -4064,13 +4064,13 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="182" fontId="25" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="23" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="25" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="23" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="182" fontId="26" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="24" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4106,60 +4106,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4168,14 +4124,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4186,35 +4139,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4580,7 +4580,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F58771A-D2E6-4840-89D0-346E4CAADD9C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FFF466C-E7F1-458C-A10F-5DECF6E08B25}">
   <sheetPr codeName="Лист1"/>
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -5059,7 +5059,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F74F0FB1-1D32-4449-85C5-84E0267B4F42}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB4D4536-1255-4465-A76D-CDD170155CFF}">
   <sheetPr codeName="Лист10"/>
   <dimension ref="A2:C11"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -5183,7 +5183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CC72E16-0189-4A95-BBA9-852AC7BA43B2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B370D0-AF89-4FF1-8CD2-65FACDEBEF38}">
   <sheetPr codeName="Лист11"/>
   <dimension ref="B2:L32"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -5196,581 +5196,620 @@
   <sheetData>
     <row r="2" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="283" t="s">
+      <c r="B3" s="270" t="s">
         <v>434</v>
       </c>
-      <c r="C3" s="271" t="s">
+      <c r="C3" s="269" t="s">
         <v>435</v>
       </c>
-      <c r="D3" s="271"/>
-      <c r="E3" s="288" t="s">
+      <c r="D3" s="269"/>
+      <c r="E3" s="258" t="s">
         <v>438</v>
       </c>
-      <c r="F3" s="288"/>
-      <c r="G3" s="288"/>
-      <c r="H3" s="288"/>
-      <c r="I3" s="277" t="s">
+      <c r="F3" s="258"/>
+      <c r="G3" s="258"/>
+      <c r="H3" s="258"/>
+      <c r="I3" s="260" t="s">
         <v>439</v>
       </c>
-      <c r="J3" s="277"/>
-      <c r="K3" s="280" t="s">
+      <c r="J3" s="260"/>
+      <c r="K3" s="263" t="s">
         <v>445</v>
       </c>
-      <c r="L3" s="254" t="s">
+      <c r="L3" s="279" t="s">
         <v>446</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B4" s="284"/>
-      <c r="C4" s="272"/>
-      <c r="D4" s="272"/>
-      <c r="E4" s="289"/>
-      <c r="F4" s="289"/>
-      <c r="G4" s="289"/>
-      <c r="H4" s="289"/>
-      <c r="I4" s="278"/>
-      <c r="J4" s="278"/>
-      <c r="K4" s="281"/>
-      <c r="L4" s="255"/>
+      <c r="B4" s="271"/>
+      <c r="C4" s="256"/>
+      <c r="D4" s="256"/>
+      <c r="E4" s="259"/>
+      <c r="F4" s="259"/>
+      <c r="G4" s="259"/>
+      <c r="H4" s="259"/>
+      <c r="I4" s="261"/>
+      <c r="J4" s="261"/>
+      <c r="K4" s="264"/>
+      <c r="L4" s="280"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B5" s="284"/>
-      <c r="C5" s="286" t="s">
+      <c r="B5" s="271"/>
+      <c r="C5" s="254" t="s">
         <v>436</v>
       </c>
-      <c r="D5" s="286" t="s">
+      <c r="D5" s="254" t="s">
         <v>437</v>
       </c>
-      <c r="E5" s="272">
+      <c r="E5" s="256">
         <v>0.5</v>
       </c>
-      <c r="F5" s="272">
+      <c r="F5" s="256">
         <v>1</v>
       </c>
-      <c r="G5" s="272">
+      <c r="G5" s="256">
         <v>3</v>
       </c>
-      <c r="H5" s="272">
+      <c r="H5" s="256">
         <v>10</v>
       </c>
-      <c r="I5" s="278"/>
-      <c r="J5" s="278"/>
-      <c r="K5" s="281"/>
-      <c r="L5" s="255"/>
+      <c r="I5" s="261"/>
+      <c r="J5" s="261"/>
+      <c r="K5" s="264"/>
+      <c r="L5" s="280"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B6" s="284"/>
-      <c r="C6" s="286"/>
-      <c r="D6" s="286"/>
-      <c r="E6" s="272"/>
-      <c r="F6" s="272"/>
-      <c r="G6" s="272"/>
-      <c r="H6" s="272"/>
-      <c r="I6" s="278"/>
-      <c r="J6" s="278"/>
-      <c r="K6" s="281"/>
-      <c r="L6" s="255"/>
+      <c r="B6" s="271"/>
+      <c r="C6" s="254"/>
+      <c r="D6" s="254"/>
+      <c r="E6" s="256"/>
+      <c r="F6" s="256"/>
+      <c r="G6" s="256"/>
+      <c r="H6" s="256"/>
+      <c r="I6" s="261"/>
+      <c r="J6" s="261"/>
+      <c r="K6" s="264"/>
+      <c r="L6" s="280"/>
     </row>
     <row r="7" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="285"/>
-      <c r="C7" s="287"/>
-      <c r="D7" s="287"/>
-      <c r="E7" s="273"/>
-      <c r="F7" s="273"/>
-      <c r="G7" s="273"/>
-      <c r="H7" s="273"/>
-      <c r="I7" s="279"/>
-      <c r="J7" s="279"/>
-      <c r="K7" s="282"/>
-      <c r="L7" s="256"/>
+      <c r="B7" s="272"/>
+      <c r="C7" s="255"/>
+      <c r="D7" s="255"/>
+      <c r="E7" s="257"/>
+      <c r="F7" s="257"/>
+      <c r="G7" s="257"/>
+      <c r="H7" s="257"/>
+      <c r="I7" s="262"/>
+      <c r="J7" s="262"/>
+      <c r="K7" s="265"/>
+      <c r="L7" s="281"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B8" s="274" t="s">
+      <c r="B8" s="266" t="s">
         <v>440</v>
       </c>
       <c r="C8" s="98">
         <v>50</v>
       </c>
-      <c r="D8" s="259">
+      <c r="D8" s="282">
         <v>5</v>
       </c>
-      <c r="E8" s="271"/>
-      <c r="F8" s="271"/>
-      <c r="G8" s="271"/>
+      <c r="E8" s="269"/>
+      <c r="F8" s="269"/>
+      <c r="G8" s="269"/>
       <c r="H8" s="92">
         <v>10</v>
       </c>
-      <c r="I8" s="269"/>
-      <c r="J8" s="270"/>
-      <c r="K8" s="259">
+      <c r="I8" s="273"/>
+      <c r="J8" s="274"/>
+      <c r="K8" s="282">
         <v>10</v>
       </c>
-      <c r="L8" s="262">
+      <c r="L8" s="285">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B9" s="275"/>
+      <c r="B9" s="267"/>
       <c r="C9" s="15">
         <v>75</v>
       </c>
-      <c r="D9" s="260"/>
-      <c r="E9" s="272"/>
-      <c r="F9" s="272"/>
-      <c r="G9" s="272"/>
+      <c r="D9" s="283"/>
+      <c r="E9" s="256"/>
+      <c r="F9" s="256"/>
+      <c r="G9" s="256"/>
       <c r="H9" s="44">
         <v>20</v>
       </c>
-      <c r="I9" s="267"/>
-      <c r="J9" s="268"/>
-      <c r="K9" s="260"/>
-      <c r="L9" s="263"/>
+      <c r="I9" s="275"/>
+      <c r="J9" s="276"/>
+      <c r="K9" s="283"/>
+      <c r="L9" s="286"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B10" s="275"/>
+      <c r="B10" s="267"/>
       <c r="C10" s="15">
         <v>100</v>
       </c>
-      <c r="D10" s="260"/>
-      <c r="E10" s="272"/>
-      <c r="F10" s="272"/>
-      <c r="G10" s="272"/>
+      <c r="D10" s="283"/>
+      <c r="E10" s="256"/>
+      <c r="F10" s="256"/>
+      <c r="G10" s="256"/>
       <c r="H10" s="44">
         <v>20</v>
       </c>
-      <c r="I10" s="267"/>
-      <c r="J10" s="268"/>
-      <c r="K10" s="260"/>
-      <c r="L10" s="263"/>
+      <c r="I10" s="275"/>
+      <c r="J10" s="276"/>
+      <c r="K10" s="283"/>
+      <c r="L10" s="286"/>
     </row>
     <row r="11" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="276"/>
+      <c r="B11" s="268"/>
       <c r="C11" s="99">
         <v>150</v>
       </c>
-      <c r="D11" s="260"/>
-      <c r="E11" s="273"/>
-      <c r="F11" s="273"/>
-      <c r="G11" s="273"/>
+      <c r="D11" s="283"/>
+      <c r="E11" s="257"/>
+      <c r="F11" s="257"/>
+      <c r="G11" s="257"/>
       <c r="H11" s="100">
         <v>30</v>
       </c>
-      <c r="I11" s="257"/>
-      <c r="J11" s="258"/>
-      <c r="K11" s="260"/>
-      <c r="L11" s="263"/>
+      <c r="I11" s="277"/>
+      <c r="J11" s="278"/>
+      <c r="K11" s="283"/>
+      <c r="L11" s="286"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B12" s="274" t="s">
+      <c r="B12" s="266" t="s">
         <v>441</v>
       </c>
       <c r="C12" s="96">
         <v>100</v>
       </c>
-      <c r="D12" s="260"/>
-      <c r="E12" s="271"/>
-      <c r="F12" s="271"/>
+      <c r="D12" s="283"/>
+      <c r="E12" s="269"/>
+      <c r="F12" s="269"/>
       <c r="G12" s="101"/>
       <c r="H12" s="102">
         <v>20</v>
       </c>
-      <c r="I12" s="269"/>
-      <c r="J12" s="270"/>
-      <c r="K12" s="260"/>
-      <c r="L12" s="263"/>
+      <c r="I12" s="273"/>
+      <c r="J12" s="274"/>
+      <c r="K12" s="283"/>
+      <c r="L12" s="286"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B13" s="275"/>
+      <c r="B13" s="267"/>
       <c r="C13" s="38">
         <v>150</v>
       </c>
-      <c r="D13" s="260"/>
-      <c r="E13" s="272"/>
-      <c r="F13" s="272"/>
+      <c r="D13" s="283"/>
+      <c r="E13" s="256"/>
+      <c r="F13" s="256"/>
       <c r="G13" s="90"/>
       <c r="H13" s="33">
         <v>30</v>
       </c>
-      <c r="I13" s="267"/>
-      <c r="J13" s="268"/>
-      <c r="K13" s="260"/>
-      <c r="L13" s="263"/>
+      <c r="I13" s="275"/>
+      <c r="J13" s="276"/>
+      <c r="K13" s="283"/>
+      <c r="L13" s="286"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B14" s="275"/>
+      <c r="B14" s="267"/>
       <c r="C14" s="38">
         <v>200</v>
       </c>
-      <c r="D14" s="260"/>
-      <c r="E14" s="272"/>
-      <c r="F14" s="272"/>
+      <c r="D14" s="283"/>
+      <c r="E14" s="256"/>
+      <c r="F14" s="256"/>
       <c r="G14" s="90"/>
       <c r="H14" s="33">
         <v>40</v>
       </c>
-      <c r="I14" s="267"/>
-      <c r="J14" s="268"/>
-      <c r="K14" s="260"/>
-      <c r="L14" s="263"/>
+      <c r="I14" s="275"/>
+      <c r="J14" s="276"/>
+      <c r="K14" s="283"/>
+      <c r="L14" s="286"/>
     </row>
     <row r="15" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="276"/>
+      <c r="B15" s="268"/>
       <c r="C15" s="99">
         <v>300</v>
       </c>
-      <c r="D15" s="260"/>
-      <c r="E15" s="273"/>
-      <c r="F15" s="273"/>
+      <c r="D15" s="283"/>
+      <c r="E15" s="257"/>
+      <c r="F15" s="257"/>
       <c r="G15" s="95">
         <v>30</v>
       </c>
       <c r="H15" s="93"/>
-      <c r="I15" s="257">
+      <c r="I15" s="277">
         <v>7</v>
       </c>
-      <c r="J15" s="258"/>
-      <c r="K15" s="260"/>
-      <c r="L15" s="263"/>
+      <c r="J15" s="278"/>
+      <c r="K15" s="283"/>
+      <c r="L15" s="286"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B16" s="274" t="s">
+      <c r="B16" s="266" t="s">
         <v>442</v>
       </c>
       <c r="C16" s="96">
         <v>200</v>
       </c>
-      <c r="D16" s="260"/>
-      <c r="E16" s="271"/>
+      <c r="D16" s="283"/>
+      <c r="E16" s="269"/>
       <c r="F16" s="101"/>
       <c r="G16" s="101"/>
       <c r="H16" s="102">
         <v>40</v>
       </c>
-      <c r="I16" s="269"/>
-      <c r="J16" s="270"/>
-      <c r="K16" s="260"/>
-      <c r="L16" s="263"/>
+      <c r="I16" s="273"/>
+      <c r="J16" s="274"/>
+      <c r="K16" s="283"/>
+      <c r="L16" s="286"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B17" s="275"/>
+      <c r="B17" s="267"/>
       <c r="C17" s="38">
         <v>300</v>
       </c>
-      <c r="D17" s="260"/>
-      <c r="E17" s="272"/>
+      <c r="D17" s="283"/>
+      <c r="E17" s="256"/>
       <c r="F17" s="90"/>
       <c r="G17" s="90">
         <v>30</v>
       </c>
       <c r="H17" s="15"/>
-      <c r="I17" s="267">
+      <c r="I17" s="275">
         <v>7</v>
       </c>
-      <c r="J17" s="268"/>
-      <c r="K17" s="260"/>
-      <c r="L17" s="263"/>
+      <c r="J17" s="276"/>
+      <c r="K17" s="283"/>
+      <c r="L17" s="286"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B18" s="275"/>
+      <c r="B18" s="267"/>
       <c r="C18" s="38">
         <v>400</v>
       </c>
-      <c r="D18" s="260"/>
-      <c r="E18" s="272"/>
+      <c r="D18" s="283"/>
+      <c r="E18" s="256"/>
       <c r="F18" s="90"/>
       <c r="G18" s="90">
         <v>40</v>
       </c>
       <c r="H18" s="15"/>
-      <c r="I18" s="267">
+      <c r="I18" s="275">
         <v>8</v>
       </c>
-      <c r="J18" s="268"/>
-      <c r="K18" s="260"/>
-      <c r="L18" s="263"/>
+      <c r="J18" s="276"/>
+      <c r="K18" s="283"/>
+      <c r="L18" s="286"/>
     </row>
     <row r="19" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="276"/>
+      <c r="B19" s="268"/>
       <c r="C19" s="99">
         <v>600</v>
       </c>
-      <c r="D19" s="260"/>
-      <c r="E19" s="273"/>
+      <c r="D19" s="283"/>
+      <c r="E19" s="257"/>
       <c r="F19" s="94">
         <v>30</v>
       </c>
       <c r="G19" s="94"/>
       <c r="H19" s="93"/>
-      <c r="I19" s="257">
+      <c r="I19" s="277">
         <v>14</v>
       </c>
-      <c r="J19" s="258"/>
-      <c r="K19" s="261"/>
-      <c r="L19" s="264"/>
+      <c r="J19" s="278"/>
+      <c r="K19" s="284"/>
+      <c r="L19" s="287"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B20" s="274" t="s">
+      <c r="B20" s="266" t="s">
         <v>442</v>
       </c>
       <c r="C20" s="96">
         <v>200</v>
       </c>
-      <c r="D20" s="260"/>
+      <c r="D20" s="283"/>
       <c r="E20" s="101"/>
       <c r="F20" s="101">
         <v>30</v>
       </c>
-      <c r="G20" s="271"/>
+      <c r="G20" s="269"/>
       <c r="H20" s="98"/>
-      <c r="I20" s="269">
+      <c r="I20" s="273">
         <v>9</v>
       </c>
-      <c r="J20" s="270"/>
-      <c r="K20" s="259">
+      <c r="J20" s="274"/>
+      <c r="K20" s="282">
         <v>20</v>
       </c>
-      <c r="L20" s="262">
+      <c r="L20" s="285">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B21" s="275"/>
+      <c r="B21" s="267"/>
       <c r="C21" s="38">
         <v>300</v>
       </c>
-      <c r="D21" s="260"/>
+      <c r="D21" s="283"/>
       <c r="E21" s="90">
         <v>30</v>
       </c>
       <c r="F21" s="90"/>
-      <c r="G21" s="272"/>
+      <c r="G21" s="256"/>
       <c r="H21" s="15"/>
-      <c r="I21" s="267">
+      <c r="I21" s="275">
         <v>14</v>
       </c>
-      <c r="J21" s="268"/>
-      <c r="K21" s="260"/>
-      <c r="L21" s="265"/>
+      <c r="J21" s="276"/>
+      <c r="K21" s="283"/>
+      <c r="L21" s="288"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B22" s="275"/>
+      <c r="B22" s="267"/>
       <c r="C22" s="38">
         <v>400</v>
       </c>
-      <c r="D22" s="260"/>
+      <c r="D22" s="283"/>
       <c r="E22" s="90">
         <v>30</v>
       </c>
       <c r="F22" s="90"/>
-      <c r="G22" s="272"/>
+      <c r="G22" s="256"/>
       <c r="H22" s="15"/>
-      <c r="I22" s="267">
+      <c r="I22" s="275">
         <v>18</v>
       </c>
-      <c r="J22" s="268"/>
-      <c r="K22" s="260"/>
-      <c r="L22" s="265"/>
+      <c r="J22" s="276"/>
+      <c r="K22" s="283"/>
+      <c r="L22" s="288"/>
     </row>
     <row r="23" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="276"/>
+      <c r="B23" s="268"/>
       <c r="C23" s="99">
         <v>600</v>
       </c>
-      <c r="D23" s="260"/>
+      <c r="D23" s="283"/>
       <c r="E23" s="94">
         <v>30</v>
       </c>
       <c r="F23" s="94"/>
-      <c r="G23" s="273"/>
+      <c r="G23" s="257"/>
       <c r="H23" s="93"/>
-      <c r="I23" s="257">
+      <c r="I23" s="277">
         <v>24</v>
       </c>
-      <c r="J23" s="258"/>
-      <c r="K23" s="261"/>
-      <c r="L23" s="266"/>
+      <c r="J23" s="278"/>
+      <c r="K23" s="284"/>
+      <c r="L23" s="289"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B24" s="274" t="s">
+      <c r="B24" s="266" t="s">
         <v>443</v>
       </c>
       <c r="C24" s="96">
         <v>600</v>
       </c>
-      <c r="D24" s="260"/>
+      <c r="D24" s="283"/>
       <c r="E24" s="97">
         <v>30</v>
       </c>
-      <c r="F24" s="271"/>
-      <c r="G24" s="271"/>
+      <c r="F24" s="269"/>
+      <c r="G24" s="269"/>
       <c r="H24" s="98"/>
-      <c r="I24" s="269">
+      <c r="I24" s="273">
         <v>27</v>
       </c>
-      <c r="J24" s="270"/>
-      <c r="K24" s="259">
+      <c r="J24" s="274"/>
+      <c r="K24" s="282">
         <v>20</v>
       </c>
-      <c r="L24" s="262">
+      <c r="L24" s="285">
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B25" s="275"/>
+      <c r="B25" s="267"/>
       <c r="C25" s="38">
         <v>800</v>
       </c>
-      <c r="D25" s="260"/>
+      <c r="D25" s="283"/>
       <c r="E25" s="91">
         <v>30</v>
       </c>
-      <c r="F25" s="272"/>
-      <c r="G25" s="272"/>
+      <c r="F25" s="256"/>
+      <c r="G25" s="256"/>
       <c r="H25" s="15"/>
-      <c r="I25" s="267">
+      <c r="I25" s="275">
         <v>25</v>
       </c>
-      <c r="J25" s="268"/>
-      <c r="K25" s="260"/>
-      <c r="L25" s="265"/>
+      <c r="J25" s="276"/>
+      <c r="K25" s="283"/>
+      <c r="L25" s="288"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B26" s="275"/>
+      <c r="B26" s="267"/>
       <c r="C26" s="38">
         <v>1000</v>
       </c>
-      <c r="D26" s="260"/>
+      <c r="D26" s="283"/>
       <c r="E26" s="91">
         <v>30</v>
       </c>
-      <c r="F26" s="272"/>
-      <c r="G26" s="272"/>
+      <c r="F26" s="256"/>
+      <c r="G26" s="256"/>
       <c r="H26" s="15"/>
-      <c r="I26" s="267">
+      <c r="I26" s="275">
         <v>20</v>
       </c>
-      <c r="J26" s="268"/>
-      <c r="K26" s="260"/>
-      <c r="L26" s="265"/>
+      <c r="J26" s="276"/>
+      <c r="K26" s="283"/>
+      <c r="L26" s="288"/>
     </row>
     <row r="27" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="276"/>
+      <c r="B27" s="268"/>
       <c r="C27" s="99">
         <v>1200</v>
       </c>
-      <c r="D27" s="260"/>
+      <c r="D27" s="283"/>
       <c r="E27" s="103">
         <v>30</v>
       </c>
-      <c r="F27" s="273"/>
-      <c r="G27" s="273"/>
+      <c r="F27" s="257"/>
+      <c r="G27" s="257"/>
       <c r="H27" s="93"/>
-      <c r="I27" s="257">
+      <c r="I27" s="277">
         <v>16</v>
       </c>
-      <c r="J27" s="258"/>
-      <c r="K27" s="260"/>
-      <c r="L27" s="265"/>
+      <c r="J27" s="278"/>
+      <c r="K27" s="283"/>
+      <c r="L27" s="288"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B28" s="274" t="s">
+      <c r="B28" s="266" t="s">
         <v>444</v>
       </c>
       <c r="C28" s="96">
         <v>600</v>
       </c>
-      <c r="D28" s="260"/>
+      <c r="D28" s="283"/>
       <c r="E28" s="97">
         <v>30</v>
       </c>
-      <c r="F28" s="271"/>
-      <c r="G28" s="271"/>
+      <c r="F28" s="269"/>
+      <c r="G28" s="269"/>
       <c r="H28" s="98"/>
-      <c r="I28" s="269">
+      <c r="I28" s="273">
         <v>27</v>
       </c>
-      <c r="J28" s="270"/>
-      <c r="K28" s="260"/>
-      <c r="L28" s="265"/>
+      <c r="J28" s="274"/>
+      <c r="K28" s="283"/>
+      <c r="L28" s="288"/>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B29" s="275"/>
+      <c r="B29" s="267"/>
       <c r="C29" s="38">
         <v>750</v>
       </c>
-      <c r="D29" s="260"/>
+      <c r="D29" s="283"/>
       <c r="E29" s="91">
         <v>30</v>
       </c>
-      <c r="F29" s="272"/>
-      <c r="G29" s="272"/>
+      <c r="F29" s="256"/>
+      <c r="G29" s="256"/>
       <c r="H29" s="15"/>
-      <c r="I29" s="267">
+      <c r="I29" s="275">
         <v>26</v>
       </c>
-      <c r="J29" s="268"/>
-      <c r="K29" s="260"/>
-      <c r="L29" s="265"/>
+      <c r="J29" s="276"/>
+      <c r="K29" s="283"/>
+      <c r="L29" s="288"/>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B30" s="275"/>
+      <c r="B30" s="267"/>
       <c r="C30" s="38">
         <v>1000</v>
       </c>
-      <c r="D30" s="260"/>
+      <c r="D30" s="283"/>
       <c r="E30" s="91">
         <v>30</v>
       </c>
-      <c r="F30" s="272"/>
-      <c r="G30" s="272"/>
+      <c r="F30" s="256"/>
+      <c r="G30" s="256"/>
       <c r="H30" s="15"/>
-      <c r="I30" s="267">
+      <c r="I30" s="275">
         <v>20</v>
       </c>
-      <c r="J30" s="268"/>
-      <c r="K30" s="260"/>
-      <c r="L30" s="265"/>
+      <c r="J30" s="276"/>
+      <c r="K30" s="283"/>
+      <c r="L30" s="288"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B31" s="275"/>
+      <c r="B31" s="267"/>
       <c r="C31" s="38">
         <v>1500</v>
       </c>
-      <c r="D31" s="260"/>
+      <c r="D31" s="283"/>
       <c r="E31" s="91">
         <v>30</v>
       </c>
-      <c r="F31" s="272"/>
-      <c r="G31" s="272"/>
+      <c r="F31" s="256"/>
+      <c r="G31" s="256"/>
       <c r="H31" s="15"/>
-      <c r="I31" s="267">
+      <c r="I31" s="275">
         <v>15</v>
       </c>
-      <c r="J31" s="268"/>
-      <c r="K31" s="260"/>
-      <c r="L31" s="265"/>
+      <c r="J31" s="276"/>
+      <c r="K31" s="283"/>
+      <c r="L31" s="288"/>
     </row>
     <row r="32" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="276"/>
+      <c r="B32" s="268"/>
       <c r="C32" s="93"/>
-      <c r="D32" s="261"/>
+      <c r="D32" s="284"/>
       <c r="E32" s="94"/>
-      <c r="F32" s="273"/>
-      <c r="G32" s="273"/>
+      <c r="F32" s="257"/>
+      <c r="G32" s="257"/>
       <c r="H32" s="93"/>
-      <c r="I32" s="257"/>
-      <c r="J32" s="258"/>
-      <c r="K32" s="261"/>
-      <c r="L32" s="266"/>
+      <c r="I32" s="277"/>
+      <c r="J32" s="278"/>
+      <c r="K32" s="284"/>
+      <c r="L32" s="289"/>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="F5:F7"/>
-    <mergeCell ref="E3:H4"/>
-    <mergeCell ref="G5:G7"/>
-    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="L3:L7"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="D8:D32"/>
+    <mergeCell ref="K8:K19"/>
+    <mergeCell ref="K20:K23"/>
+    <mergeCell ref="K24:K32"/>
+    <mergeCell ref="L8:L19"/>
+    <mergeCell ref="L20:L23"/>
+    <mergeCell ref="L24:L32"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="F24:F27"/>
+    <mergeCell ref="F28:F32"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="G20:G23"/>
+    <mergeCell ref="G24:G27"/>
+    <mergeCell ref="G28:G32"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B32"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="E16:E19"/>
     <mergeCell ref="I3:J7"/>
     <mergeCell ref="K3:K7"/>
     <mergeCell ref="B8:B11"/>
@@ -5781,51 +5820,12 @@
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="C3:D4"/>
     <mergeCell ref="C5:C7"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B32"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="F24:F27"/>
-    <mergeCell ref="F28:F32"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="G20:G23"/>
-    <mergeCell ref="G24:G27"/>
-    <mergeCell ref="G28:G32"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="L3:L7"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="D8:D32"/>
-    <mergeCell ref="K8:K19"/>
-    <mergeCell ref="K20:K23"/>
-    <mergeCell ref="K24:K32"/>
-    <mergeCell ref="L8:L19"/>
-    <mergeCell ref="L20:L23"/>
-    <mergeCell ref="L24:L32"/>
-    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="E3:H4"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="H5:H7"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="85" orientation="portrait" r:id="rId1"/>
@@ -5833,7 +5833,8 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B495BE74-6474-4C14-A79F-F5EC806EB1E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36348D1A-404C-4220-BD1E-353B721C8A2B}">
+  <sheetPr codeName="Лист12"/>
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -6126,7 +6127,8 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB86133C-D7DD-4EA1-8EF7-67B8C194A0C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75D4DE35-7328-4EA5-8411-7B3098D70ED4}">
+  <sheetPr codeName="Лист13"/>
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -6304,7 +6306,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92EA8145-53D5-4538-922E-58462E5A6AD9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9DE87C7-8B15-49E6-8F80-0E1ABE0B5202}">
   <sheetPr codeName="Лист2"/>
   <dimension ref="A1:K82"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -7807,7 +7809,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97251408-9674-4151-A6AC-297AB0F87392}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576A4536-36B8-484E-BA2B-13A68D8E51C7}">
   <sheetPr codeName="Лист3"/>
   <dimension ref="A1:K272"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -9156,7 +9158,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E36C285-BE2D-48C4-9898-B6A62A301D6A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E42E220-D35C-4A24-A836-F2D4EB04706D}">
   <sheetPr codeName="Лист4"/>
   <dimension ref="A1:S454"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -20117,7 +20119,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11D9B79D-73FA-47F3-BCCD-FC8F3077A97C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8535B297-B813-4CBD-9D27-3E847A750622}">
   <sheetPr codeName="Лист5"/>
   <dimension ref="A1:P26"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -20812,7 +20814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938BBFBA-670D-4068-B550-7C614D69B968}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FED76680-BCB1-44CB-A601-471C0227000E}">
   <sheetPr codeName="Лист6"/>
   <dimension ref="A1:E59"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -21435,7 +21437,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5906A8-CD6B-440A-88B0-C25E54BBF18C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67A5C948-BD94-487A-955B-28FDB758389C}">
   <sheetPr codeName="Лист7"/>
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -21480,7 +21482,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE39ED22-E59F-4A2D-AC28-3F8073AE0E2B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A9063C-CDB4-4CD7-850A-C5399340D177}">
   <sheetPr codeName="Лист8"/>
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -21740,7 +21742,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{875D5023-E29F-4F0F-8120-9F03A5A27CCA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DCDDA8C-A328-4C39-BA7A-587A721210D1}">
   <sheetPr codeName="Лист9"/>
   <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>

</xml_diff>